<commit_message>
GRCW-1080; Updated CSVs for next draft. RTTBC26 Week 17 Noms (SA)
</commit_message>
<xml_diff>
--- a/pdf/RTTBC26-Schedule-by-Division.xlsx
+++ b/pdf/RTTBC26-Schedule-by-Division.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/299f8723705ec823/Webmaster/gallop-racing/pdf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1608" documentId="8_{DAECCBE5-FF72-4188-B2F1-1541968A3FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2412A872-B8A8-4258-A052-180374A1C0D7}"/>
+  <xr:revisionPtr revIDLastSave="1609" documentId="8_{DAECCBE5-FF72-4188-B2F1-1541968A3FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40FDFAB2-E02A-49F5-B33A-F57978DA2791}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{EAD27B02-19FE-4D48-9014-ED6E24DB84F0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{EAD27B02-19FE-4D48-9014-ED6E24DB84F0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="112">
   <si>
     <t>9 Furlongs</t>
   </si>
@@ -228,9 +228,6 @@
   </si>
   <si>
     <t>Chillingworth S.-G3</t>
-  </si>
-  <si>
-    <t>Woodward S.-G2</t>
   </si>
   <si>
     <t>Gallant Bloom H.-G2</t>
@@ -926,77 +923,119 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1004,22 +1043,13 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1034,95 +1064,62 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1144,10 +1141,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1448,60 +1441,60 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1783450-6415-4D0D-A0B8-DEE615502A89}">
   <dimension ref="A1:I43"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="4.28515625" style="28" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" style="28" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="36" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="32.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="32.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="34.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="32.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="34.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.6640625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="117"/>
-      <c r="B1" s="117"/>
-      <c r="C1" s="132" t="s">
+    <row r="1" spans="1:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.65">
+      <c r="A1" s="69"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="84" t="s">
+        <v>87</v>
+      </c>
+      <c r="D1" s="84"/>
+      <c r="E1" s="84"/>
+      <c r="F1" s="84"/>
+      <c r="G1" s="84"/>
+      <c r="H1" s="84"/>
+      <c r="I1" s="84"/>
+    </row>
+    <row r="2" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="A2" s="86" t="s">
         <v>88</v>
-      </c>
-      <c r="D1" s="132"/>
-      <c r="E1" s="132"/>
-      <c r="F1" s="132"/>
-      <c r="G1" s="132"/>
-      <c r="H1" s="132"/>
-      <c r="I1" s="132"/>
-    </row>
-    <row r="2" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A2" s="133" t="s">
-        <v>89</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="24" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D2" s="24" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E2" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="F2" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="G2" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="H2" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="G2" s="24" t="s">
-        <v>82</v>
-      </c>
-      <c r="H2" s="24" t="s">
+      <c r="I2" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="I2" s="24" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="133"/>
+    </row>
+    <row r="3" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="86"/>
       <c r="B3" s="27"/>
       <c r="C3" s="25" t="s">
         <v>5</v>
@@ -1525,9 +1518,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A4" s="133"/>
-      <c r="B4" s="118">
+    <row r="4" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="A4" s="86"/>
+      <c r="B4" s="82">
         <v>1</v>
       </c>
       <c r="C4" s="21" t="s">
@@ -1536,67 +1529,67 @@
       <c r="D4" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="76"/>
-      <c r="F4" s="76"/>
-      <c r="G4" s="71" t="s">
+      <c r="E4" s="70"/>
+      <c r="F4" s="70"/>
+      <c r="G4" s="94" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="84" t="s">
-        <v>90</v>
+      <c r="H4" s="91" t="s">
+        <v>89</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="133"/>
-      <c r="B5" s="119"/>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="86"/>
+      <c r="B5" s="93"/>
       <c r="C5" s="11" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="64" t="s">
-        <v>104</v>
-      </c>
-      <c r="E5" s="77"/>
-      <c r="F5" s="77"/>
-      <c r="G5" s="73"/>
-      <c r="H5" s="85"/>
+        <v>103</v>
+      </c>
+      <c r="E5" s="71"/>
+      <c r="F5" s="71"/>
+      <c r="G5" s="95"/>
+      <c r="H5" s="92"/>
       <c r="I5" s="65" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="133"/>
-      <c r="B6" s="78">
+    <row r="6" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="86"/>
+      <c r="B6" s="87">
         <v>2</v>
       </c>
-      <c r="C6" s="76"/>
+      <c r="C6" s="70"/>
       <c r="D6" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="76"/>
-      <c r="F6" s="76"/>
-      <c r="G6" s="74" t="s">
+      <c r="E6" s="70"/>
+      <c r="F6" s="70"/>
+      <c r="G6" s="89" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="80"/>
-      <c r="I6" s="76"/>
-    </row>
-    <row r="7" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="133"/>
-      <c r="B7" s="79"/>
-      <c r="C7" s="77"/>
+      <c r="H6" s="131"/>
+      <c r="I6" s="70"/>
+    </row>
+    <row r="7" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="86"/>
+      <c r="B7" s="88"/>
+      <c r="C7" s="71"/>
       <c r="D7" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="E7" s="77"/>
-      <c r="F7" s="77"/>
-      <c r="G7" s="75"/>
-      <c r="H7" s="81"/>
-      <c r="I7" s="77"/>
-    </row>
-    <row r="8" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="133"/>
+        <v>99</v>
+      </c>
+      <c r="E7" s="71"/>
+      <c r="F7" s="71"/>
+      <c r="G7" s="90"/>
+      <c r="H7" s="132"/>
+      <c r="I7" s="71"/>
+    </row>
+    <row r="8" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="86"/>
       <c r="B8" s="63">
         <v>3</v>
       </c>
@@ -1608,46 +1601,46 @@
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="38" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I8" s="3"/>
     </row>
-    <row r="9" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="133"/>
-      <c r="B9" s="118">
+    <row r="9" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="86"/>
+      <c r="B9" s="82">
         <v>4</v>
       </c>
-      <c r="C9" s="71" t="s">
+      <c r="C9" s="94" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="86" t="s">
+      <c r="D9" s="116" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="76"/>
-      <c r="F9" s="88"/>
+      <c r="E9" s="70"/>
+      <c r="F9" s="126"/>
       <c r="G9" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H9" s="128"/>
+      <c r="I9" s="89" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" s="35" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="86"/>
+      <c r="B10" s="93"/>
+      <c r="C10" s="95"/>
+      <c r="D10" s="118"/>
+      <c r="E10" s="71"/>
+      <c r="F10" s="127"/>
+      <c r="G10" s="42" t="s">
         <v>110</v>
       </c>
-      <c r="H9" s="90"/>
-      <c r="I9" s="74" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" s="35" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="133"/>
-      <c r="B10" s="119"/>
-      <c r="C10" s="73"/>
-      <c r="D10" s="87"/>
-      <c r="E10" s="77"/>
-      <c r="F10" s="89"/>
-      <c r="G10" s="42" t="s">
-        <v>111</v>
-      </c>
-      <c r="H10" s="91"/>
-      <c r="I10" s="75"/>
-    </row>
-    <row r="11" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="133"/>
+      <c r="H10" s="129"/>
+      <c r="I10" s="90"/>
+    </row>
+    <row r="11" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="86"/>
       <c r="B11" s="56">
         <v>5</v>
       </c>
@@ -1665,119 +1658,119 @@
       </c>
       <c r="I11" s="37"/>
     </row>
-    <row r="12" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="133"/>
-      <c r="B12" s="78">
+    <row r="12" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="86"/>
+      <c r="B12" s="87">
         <v>6</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="74" t="s">
+      <c r="D12" s="89" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="82"/>
-      <c r="F12" s="82"/>
-      <c r="G12" s="76"/>
-      <c r="H12" s="74" t="s">
+      <c r="E12" s="133"/>
+      <c r="F12" s="133"/>
+      <c r="G12" s="70"/>
+      <c r="H12" s="89" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="76"/>
-    </row>
-    <row r="13" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="133"/>
-      <c r="B13" s="79"/>
+      <c r="I12" s="70"/>
+    </row>
+    <row r="13" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="86"/>
+      <c r="B13" s="88"/>
       <c r="C13" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="75"/>
-      <c r="E13" s="83"/>
-      <c r="F13" s="83"/>
-      <c r="G13" s="77"/>
-      <c r="H13" s="75"/>
-      <c r="I13" s="77"/>
-    </row>
-    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="133"/>
-      <c r="B14" s="118">
+      <c r="D13" s="90"/>
+      <c r="E13" s="134"/>
+      <c r="F13" s="134"/>
+      <c r="G13" s="71"/>
+      <c r="H13" s="90"/>
+      <c r="I13" s="71"/>
+    </row>
+    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="86"/>
+      <c r="B14" s="82">
         <v>7</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="84" t="s">
-        <v>109</v>
-      </c>
-      <c r="E14" s="76"/>
-      <c r="F14" s="76"/>
-      <c r="G14" s="69" t="s">
+      <c r="D14" s="91" t="s">
+        <v>108</v>
+      </c>
+      <c r="E14" s="70"/>
+      <c r="F14" s="70"/>
+      <c r="G14" s="119" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="84"/>
-      <c r="I14" s="84"/>
-    </row>
-    <row r="15" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="133"/>
-      <c r="B15" s="119"/>
+      <c r="H14" s="91"/>
+      <c r="I14" s="91"/>
+    </row>
+    <row r="15" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="86"/>
+      <c r="B15" s="93"/>
       <c r="C15" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="85"/>
-      <c r="E15" s="77"/>
-      <c r="F15" s="77"/>
-      <c r="G15" s="70"/>
-      <c r="H15" s="85"/>
-      <c r="I15" s="85"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="133"/>
-      <c r="B16" s="118">
+      <c r="D15" s="92"/>
+      <c r="E15" s="71"/>
+      <c r="F15" s="71"/>
+      <c r="G15" s="121"/>
+      <c r="H15" s="92"/>
+      <c r="I15" s="92"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="86"/>
+      <c r="B16" s="82">
         <v>8</v>
       </c>
-      <c r="C16" s="106"/>
+      <c r="C16" s="96"/>
       <c r="D16" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="120"/>
-      <c r="F16" s="76"/>
-      <c r="G16" s="69"/>
-      <c r="H16" s="106" t="s">
+      <c r="E16" s="99"/>
+      <c r="F16" s="70"/>
+      <c r="G16" s="119"/>
+      <c r="H16" s="96" t="s">
         <v>27</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A17" s="133"/>
-      <c r="B17" s="123"/>
-      <c r="C17" s="107"/>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="A17" s="86"/>
+      <c r="B17" s="83"/>
+      <c r="C17" s="97"/>
       <c r="D17" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="121"/>
-      <c r="F17" s="92"/>
-      <c r="G17" s="109"/>
-      <c r="H17" s="107"/>
+      <c r="E17" s="100"/>
+      <c r="F17" s="79"/>
+      <c r="G17" s="120"/>
+      <c r="H17" s="97"/>
       <c r="I17" s="17" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="133"/>
-      <c r="B18" s="119"/>
-      <c r="C18" s="108"/>
+    <row r="18" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="86"/>
+      <c r="B18" s="93"/>
+      <c r="C18" s="98"/>
       <c r="D18" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="122"/>
-      <c r="F18" s="77"/>
-      <c r="G18" s="70"/>
-      <c r="H18" s="108"/>
+      <c r="E18" s="101"/>
+      <c r="F18" s="71"/>
+      <c r="G18" s="121"/>
+      <c r="H18" s="98"/>
       <c r="I18" s="47"/>
     </row>
-    <row r="19" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="133"/>
+    <row r="19" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="86"/>
       <c r="B19" s="56">
         <v>9</v>
       </c>
@@ -1799,42 +1792,42 @@
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A20" s="133"/>
-      <c r="B20" s="78">
+    <row r="20" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="A20" s="86"/>
+      <c r="B20" s="87">
         <v>10</v>
       </c>
       <c r="C20" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="76"/>
-      <c r="E20" s="74" t="s">
+      <c r="D20" s="70"/>
+      <c r="E20" s="89" t="s">
         <v>39</v>
       </c>
-      <c r="F20" s="74" t="s">
+      <c r="F20" s="89" t="s">
         <v>38</v>
       </c>
-      <c r="G20" s="76"/>
-      <c r="H20" s="97" t="s">
-        <v>94</v>
-      </c>
-      <c r="I20" s="76"/>
-    </row>
-    <row r="21" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="133"/>
-      <c r="B21" s="79"/>
+      <c r="G20" s="70"/>
+      <c r="H20" s="103" t="s">
+        <v>93</v>
+      </c>
+      <c r="I20" s="70"/>
+    </row>
+    <row r="21" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="86"/>
+      <c r="B21" s="88"/>
       <c r="C21" s="54" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="77"/>
-      <c r="E21" s="75"/>
-      <c r="F21" s="75"/>
-      <c r="G21" s="77"/>
-      <c r="H21" s="98"/>
-      <c r="I21" s="77"/>
-    </row>
-    <row r="22" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="133"/>
+      <c r="D21" s="71"/>
+      <c r="E21" s="90"/>
+      <c r="F21" s="90"/>
+      <c r="G21" s="71"/>
+      <c r="H21" s="104"/>
+      <c r="I21" s="71"/>
+    </row>
+    <row r="22" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="86"/>
       <c r="B22" s="56">
         <v>11</v>
       </c>
@@ -1850,8 +1843,8 @@
       </c>
       <c r="I22" s="4"/>
     </row>
-    <row r="23" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="133"/>
+    <row r="23" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="86"/>
       <c r="B23" s="62">
         <v>12</v>
       </c>
@@ -1867,101 +1860,101 @@
       <c r="H23" s="48"/>
       <c r="I23" s="46"/>
     </row>
-    <row r="24" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A24" s="133"/>
-      <c r="B24" s="78">
+    <row r="24" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="A24" s="86"/>
+      <c r="B24" s="87">
         <v>13</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D24" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="E24" s="97"/>
-      <c r="F24" s="111"/>
+      <c r="E24" s="103"/>
+      <c r="F24" s="109"/>
       <c r="G24" s="36" t="s">
         <v>48</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="I24" s="76"/>
-    </row>
-    <row r="25" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A25" s="133"/>
-      <c r="B25" s="100"/>
+        <v>96</v>
+      </c>
+      <c r="I24" s="70"/>
+    </row>
+    <row r="25" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="A25" s="86"/>
+      <c r="B25" s="102"/>
       <c r="C25" s="9" t="s">
         <v>42</v>
       </c>
       <c r="D25" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="E25" s="116"/>
-      <c r="F25" s="112"/>
+      <c r="E25" s="111"/>
+      <c r="F25" s="123"/>
       <c r="G25" s="19" t="s">
         <v>45</v>
       </c>
       <c r="H25" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="I25" s="92"/>
-    </row>
-    <row r="26" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="133"/>
-      <c r="B26" s="79"/>
+      <c r="I25" s="79"/>
+    </row>
+    <row r="26" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A26" s="86"/>
+      <c r="B26" s="88"/>
       <c r="C26" s="47"/>
       <c r="D26" s="49"/>
-      <c r="E26" s="98"/>
-      <c r="F26" s="113"/>
+      <c r="E26" s="104"/>
+      <c r="F26" s="110"/>
       <c r="G26" s="20" t="s">
         <v>44</v>
       </c>
       <c r="H26" s="42"/>
-      <c r="I26" s="77"/>
-    </row>
-    <row r="27" spans="1:9" ht="21" x14ac:dyDescent="0.25">
-      <c r="A27" s="133"/>
-      <c r="B27" s="78">
+      <c r="I26" s="71"/>
+    </row>
+    <row r="27" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+      <c r="A27" s="86"/>
+      <c r="B27" s="87">
         <v>14</v>
       </c>
-      <c r="C27" s="93"/>
-      <c r="D27" s="111"/>
+      <c r="C27" s="107"/>
+      <c r="D27" s="109"/>
       <c r="E27" s="29" t="s">
         <v>53</v>
       </c>
       <c r="F27" s="51" t="s">
         <v>52</v>
       </c>
-      <c r="G27" s="93"/>
-      <c r="H27" s="95" t="s">
-        <v>96</v>
-      </c>
-      <c r="I27" s="76"/>
-    </row>
-    <row r="28" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="133"/>
-      <c r="B28" s="79"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="113"/>
+      <c r="G27" s="107"/>
+      <c r="H27" s="124" t="s">
+        <v>95</v>
+      </c>
+      <c r="I27" s="70"/>
+    </row>
+    <row r="28" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A28" s="86"/>
+      <c r="B28" s="88"/>
+      <c r="C28" s="108"/>
+      <c r="D28" s="110"/>
       <c r="E28" s="53" t="s">
         <v>55</v>
       </c>
       <c r="F28" s="52" t="s">
         <v>54</v>
       </c>
-      <c r="G28" s="94"/>
-      <c r="H28" s="96"/>
-      <c r="I28" s="77"/>
-    </row>
-    <row r="29" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="133"/>
+      <c r="G28" s="108"/>
+      <c r="H28" s="125"/>
+      <c r="I28" s="71"/>
+    </row>
+    <row r="29" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="86"/>
       <c r="B29" s="66">
         <v>15</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E29" s="31" t="s">
         <v>56</v>
@@ -1971,169 +1964,167 @@
       </c>
       <c r="G29" s="2"/>
       <c r="H29" s="68" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I29" s="2"/>
     </row>
-    <row r="30" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="133"/>
-      <c r="B30" s="78">
+    <row r="30" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="86"/>
+      <c r="B30" s="87">
         <v>16</v>
       </c>
       <c r="C30" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="D30" s="97" t="s">
+      <c r="D30" s="103" t="s">
         <v>58</v>
       </c>
-      <c r="E30" s="114"/>
-      <c r="F30" s="76"/>
-      <c r="G30" s="76"/>
-      <c r="H30" s="74" t="s">
+      <c r="E30" s="105"/>
+      <c r="F30" s="70"/>
+      <c r="G30" s="70"/>
+      <c r="H30" s="89" t="s">
         <v>61</v>
       </c>
-      <c r="I30" s="84" t="s">
+      <c r="I30" s="91" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="133"/>
-      <c r="B31" s="79"/>
+    <row r="31" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A31" s="86"/>
+      <c r="B31" s="88"/>
       <c r="C31" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="D31" s="98"/>
-      <c r="E31" s="115"/>
-      <c r="F31" s="77"/>
-      <c r="G31" s="77"/>
-      <c r="H31" s="75"/>
-      <c r="I31" s="85"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="133"/>
-      <c r="B32" s="118">
+      <c r="D31" s="104"/>
+      <c r="E31" s="106"/>
+      <c r="F31" s="71"/>
+      <c r="G31" s="71"/>
+      <c r="H31" s="90"/>
+      <c r="I31" s="92"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32" s="86"/>
+      <c r="B32" s="82">
         <v>17</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="5"/>
+      <c r="D32" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E32" s="70"/>
+      <c r="F32" s="70"/>
+      <c r="G32" s="80" t="s">
+        <v>68</v>
+      </c>
+      <c r="H32" s="91" t="s">
         <v>64</v>
       </c>
-      <c r="D32" s="36" t="s">
-        <v>70</v>
-      </c>
-      <c r="E32" s="76"/>
-      <c r="F32" s="76"/>
-      <c r="G32" s="130" t="s">
-        <v>69</v>
-      </c>
-      <c r="H32" s="84" t="s">
+      <c r="I32" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="I32" s="7" t="s">
+    </row>
+    <row r="33" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="A33" s="86"/>
+      <c r="B33" s="83"/>
+      <c r="C33" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="D33" s="39" t="s">
+        <v>100</v>
+      </c>
+      <c r="E33" s="79"/>
+      <c r="F33" s="79"/>
+      <c r="G33" s="81"/>
+      <c r="H33" s="122"/>
+      <c r="I33" s="41" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A33" s="133"/>
-      <c r="B33" s="123"/>
-      <c r="C33" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="D33" s="39" t="s">
-        <v>101</v>
-      </c>
-      <c r="E33" s="92"/>
-      <c r="F33" s="92"/>
-      <c r="G33" s="131"/>
-      <c r="H33" s="110"/>
-      <c r="I33" s="41" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="133"/>
-      <c r="B34" s="123"/>
+    <row r="34" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="86"/>
+      <c r="B34" s="83"/>
       <c r="C34" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="D34" s="134" t="s">
+      <c r="D34" s="85" t="s">
+        <v>74</v>
+      </c>
+      <c r="E34" s="79"/>
+      <c r="F34" s="79"/>
+      <c r="G34" s="81"/>
+      <c r="H34" s="122"/>
+      <c r="I34" s="115"/>
+    </row>
+    <row r="35" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A35" s="86"/>
+      <c r="B35" s="83"/>
+      <c r="C35" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="D35" s="85"/>
+      <c r="E35" s="79"/>
+      <c r="F35" s="79"/>
+      <c r="G35" s="81"/>
+      <c r="H35" s="122"/>
+      <c r="I35" s="115"/>
+    </row>
+    <row r="36" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="A36" s="86"/>
+      <c r="B36" s="87">
+        <v>18</v>
+      </c>
+      <c r="C36" s="112"/>
+      <c r="D36" s="94" t="s">
+        <v>105</v>
+      </c>
+      <c r="E36" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="F36" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="G36" s="70"/>
+      <c r="H36" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="E34" s="92"/>
-      <c r="F34" s="92"/>
-      <c r="G34" s="131"/>
-      <c r="H34" s="110"/>
-      <c r="I34" s="104"/>
-    </row>
-    <row r="35" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="133"/>
-      <c r="B35" s="123"/>
-      <c r="C35" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="D35" s="134"/>
-      <c r="E35" s="92"/>
-      <c r="F35" s="92"/>
-      <c r="G35" s="131"/>
-      <c r="H35" s="110"/>
-      <c r="I35" s="104"/>
-    </row>
-    <row r="36" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A36" s="133"/>
-      <c r="B36" s="78">
-        <v>18</v>
-      </c>
-      <c r="C36" s="101"/>
-      <c r="D36" s="71" t="s">
-        <v>106</v>
-      </c>
-      <c r="E36" s="18" t="s">
+      <c r="I36" s="116" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="A37" s="86"/>
+      <c r="B37" s="102"/>
+      <c r="C37" s="113"/>
+      <c r="D37" s="130"/>
+      <c r="E37" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="F37" s="40" t="s">
         <v>72</v>
       </c>
-      <c r="F36" s="18" t="s">
-        <v>108</v>
-      </c>
-      <c r="G36" s="76"/>
-      <c r="H36" s="32" t="s">
-        <v>76</v>
-      </c>
-      <c r="I36" s="86" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A37" s="133"/>
-      <c r="B37" s="100"/>
-      <c r="C37" s="102"/>
-      <c r="D37" s="72"/>
-      <c r="E37" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="F37" s="40" t="s">
-        <v>73</v>
-      </c>
-      <c r="G37" s="92"/>
+      <c r="G37" s="79"/>
       <c r="H37" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I37" s="105"/>
-    </row>
-    <row r="38" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="133"/>
-      <c r="B38" s="79"/>
-      <c r="C38" s="103"/>
-      <c r="D38" s="73"/>
+      <c r="I37" s="117"/>
+    </row>
+    <row r="38" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A38" s="86"/>
+      <c r="B38" s="88"/>
+      <c r="C38" s="114"/>
+      <c r="D38" s="95"/>
       <c r="E38" s="20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F38" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="G38" s="77"/>
+        <v>97</v>
+      </c>
+      <c r="G38" s="71"/>
       <c r="H38" s="33"/>
-      <c r="I38" s="87"/>
-    </row>
-    <row r="39" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="133"/>
+      <c r="I38" s="118"/>
+    </row>
+    <row r="39" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A39" s="86"/>
       <c r="B39" s="63">
         <v>20</v>
       </c>
@@ -2143,31 +2134,31 @@
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="117"/>
-      <c r="B40" s="99" t="s">
-        <v>87</v>
-      </c>
-      <c r="C40" s="99"/>
-      <c r="D40" s="99"/>
-      <c r="E40" s="99"/>
-      <c r="F40" s="99"/>
-      <c r="G40" s="99"/>
-      <c r="H40" s="99"/>
-      <c r="I40" s="129"/>
-    </row>
-    <row r="41" spans="1:9" s="14" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="117"/>
+        <v>92</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A40" s="69"/>
+      <c r="B40" s="77" t="s">
+        <v>86</v>
+      </c>
+      <c r="C40" s="77"/>
+      <c r="D40" s="77"/>
+      <c r="E40" s="77"/>
+      <c r="F40" s="77"/>
+      <c r="G40" s="77"/>
+      <c r="H40" s="77"/>
+      <c r="I40" s="78"/>
+    </row>
+    <row r="41" spans="1:9" s="14" customFormat="1" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A41" s="69"/>
       <c r="B41" s="16"/>
       <c r="C41" s="15">
         <f>COUNTIF(C4:C39, "&lt;&gt;")</f>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D41" s="15">
         <f>COUNTIF(D4:D39, "&lt;&gt;")</f>
@@ -2194,37 +2185,104 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="117"/>
-      <c r="B42" s="99" t="str">
+    <row r="42" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A42" s="69"/>
+      <c r="B42" s="77" t="str">
         <f>SUM(C41:I41) &amp; " Total Races (Prior to Breeders' Cup Weekend)"</f>
-        <v>95 Total Races (Prior to Breeders' Cup Weekend)</v>
-      </c>
-      <c r="C42" s="99"/>
-      <c r="D42" s="99"/>
-      <c r="E42" s="99"/>
-      <c r="F42" s="99"/>
-      <c r="G42" s="99"/>
-      <c r="H42" s="99"/>
-      <c r="I42" s="99"/>
-    </row>
-    <row r="43" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="117"/>
-      <c r="B43" s="124" t="s">
+        <v>94 Total Races (Prior to Breeders' Cup Weekend)</v>
+      </c>
+      <c r="C42" s="77"/>
+      <c r="D42" s="77"/>
+      <c r="E42" s="77"/>
+      <c r="F42" s="77"/>
+      <c r="G42" s="77"/>
+      <c r="H42" s="77"/>
+      <c r="I42" s="77"/>
+    </row>
+    <row r="43" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A43" s="69"/>
+      <c r="B43" s="72" t="s">
+        <v>84</v>
+      </c>
+      <c r="C43" s="72"/>
+      <c r="D43" s="72"/>
+      <c r="E43" s="73"/>
+      <c r="F43" s="74" t="s">
         <v>85</v>
       </c>
-      <c r="C43" s="124"/>
-      <c r="D43" s="124"/>
-      <c r="E43" s="125"/>
-      <c r="F43" s="126" t="s">
-        <v>86</v>
-      </c>
-      <c r="G43" s="127"/>
-      <c r="H43" s="127"/>
-      <c r="I43" s="128"/>
+      <c r="G43" s="75"/>
+      <c r="H43" s="75"/>
+      <c r="I43" s="76"/>
     </row>
   </sheetData>
   <mergeCells count="83">
+    <mergeCell ref="D36:D38"/>
+    <mergeCell ref="H30:H31"/>
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="G12:G13"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="I24:I26"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="H27:H28"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="I12:I13"/>
+    <mergeCell ref="H20:H21"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="B42:I42"/>
+    <mergeCell ref="G36:G38"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="C36:C38"/>
+    <mergeCell ref="I34:I35"/>
+    <mergeCell ref="I36:I38"/>
+    <mergeCell ref="H16:H18"/>
+    <mergeCell ref="G16:G18"/>
+    <mergeCell ref="F16:F18"/>
+    <mergeCell ref="H32:H35"/>
+    <mergeCell ref="F24:F26"/>
+    <mergeCell ref="I30:I31"/>
+    <mergeCell ref="G30:G31"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="F30:F31"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="A40:A43"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="F4:F5"/>
@@ -2241,73 +2299,6 @@
     <mergeCell ref="A2:A39"/>
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="D20:D21"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="A40:A43"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="E16:E18"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="H20:H21"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="B42:I42"/>
-    <mergeCell ref="G36:G38"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="C36:C38"/>
-    <mergeCell ref="I34:I35"/>
-    <mergeCell ref="I36:I38"/>
-    <mergeCell ref="H16:H18"/>
-    <mergeCell ref="G16:G18"/>
-    <mergeCell ref="F16:F18"/>
-    <mergeCell ref="H32:H35"/>
-    <mergeCell ref="F24:F26"/>
-    <mergeCell ref="I30:I31"/>
-    <mergeCell ref="G30:G31"/>
-    <mergeCell ref="F30:F31"/>
-    <mergeCell ref="I24:I26"/>
-    <mergeCell ref="G27:G28"/>
-    <mergeCell ref="H27:H28"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="H12:H13"/>
-    <mergeCell ref="I12:I13"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="D36:D38"/>
-    <mergeCell ref="H30:H31"/>
-    <mergeCell ref="I20:I21"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="G12:G13"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="51" fitToHeight="10" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
QA Fixes; GRCW-1084; RTTBC26 Week 17 Results (Sat); Jockey Updates for Week 17 PDF; GRCW-1014
</commit_message>
<xml_diff>
--- a/pdf/RTTBC26-Schedule-by-Division.xlsx
+++ b/pdf/RTTBC26-Schedule-by-Division.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/299f8723705ec823/Webmaster/gallop-racing/pdf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1609" documentId="8_{DAECCBE5-FF72-4188-B2F1-1541968A3FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40FDFAB2-E02A-49F5-B33A-F57978DA2791}"/>
+  <xr:revisionPtr revIDLastSave="1622" documentId="8_{DAECCBE5-FF72-4188-B2F1-1541968A3FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{750E098A-DDA0-4D5B-9FEF-95D99D67400B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{EAD27B02-19FE-4D48-9014-ED6E24DB84F0}"/>
   </bookViews>
@@ -723,7 +723,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="135">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -923,203 +923,209 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1141,6 +1147,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1440,7 +1450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1783450-6415-4D0D-A0B8-DEE615502A89}">
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="4.33203125" style="28" bestFit="1" customWidth="1"/>
@@ -1454,20 +1464,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="69"/>
-      <c r="B1" s="69"/>
-      <c r="C1" s="84" t="s">
+      <c r="A1" s="117"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="134" t="s">
         <v>87</v>
       </c>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="84"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
+      <c r="D1" s="134"/>
+      <c r="E1" s="134"/>
+      <c r="F1" s="134"/>
+      <c r="G1" s="134"/>
+      <c r="H1" s="134"/>
+      <c r="I1" s="134"/>
     </row>
     <row r="2" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A2" s="86" t="s">
+      <c r="A2" s="135" t="s">
         <v>88</v>
       </c>
       <c r="B2" s="26"/>
@@ -1494,7 +1504,7 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="86"/>
+      <c r="A3" s="135"/>
       <c r="B3" s="27"/>
       <c r="C3" s="25" t="s">
         <v>5</v>
@@ -1519,8 +1529,8 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A4" s="86"/>
-      <c r="B4" s="82">
+      <c r="A4" s="135"/>
+      <c r="B4" s="118">
         <v>1</v>
       </c>
       <c r="C4" s="21" t="s">
@@ -1529,12 +1539,12 @@
       <c r="D4" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="70"/>
-      <c r="F4" s="70"/>
-      <c r="G4" s="94" t="s">
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
+      <c r="G4" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="91" t="s">
+      <c r="H4" s="85" t="s">
         <v>89</v>
       </c>
       <c r="I4" s="8" t="s">
@@ -1542,54 +1552,54 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="86"/>
-      <c r="B5" s="93"/>
+      <c r="A5" s="135"/>
+      <c r="B5" s="119"/>
       <c r="C5" s="11" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="64" t="s">
         <v>103</v>
       </c>
-      <c r="E5" s="71"/>
-      <c r="F5" s="71"/>
-      <c r="G5" s="95"/>
-      <c r="H5" s="92"/>
+      <c r="E5" s="78"/>
+      <c r="F5" s="78"/>
+      <c r="G5" s="74"/>
+      <c r="H5" s="86"/>
       <c r="I5" s="65" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="86"/>
-      <c r="B6" s="87">
+      <c r="A6" s="135"/>
+      <c r="B6" s="79">
         <v>2</v>
       </c>
-      <c r="C6" s="70"/>
+      <c r="C6" s="77"/>
       <c r="D6" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="70"/>
-      <c r="F6" s="70"/>
-      <c r="G6" s="89" t="s">
+      <c r="E6" s="77"/>
+      <c r="F6" s="77"/>
+      <c r="G6" s="75" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="131"/>
-      <c r="I6" s="70"/>
+      <c r="H6" s="81"/>
+      <c r="I6" s="77"/>
     </row>
     <row r="7" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="86"/>
-      <c r="B7" s="88"/>
-      <c r="C7" s="71"/>
+      <c r="A7" s="135"/>
+      <c r="B7" s="80"/>
+      <c r="C7" s="78"/>
       <c r="D7" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="E7" s="71"/>
-      <c r="F7" s="71"/>
-      <c r="G7" s="90"/>
-      <c r="H7" s="132"/>
-      <c r="I7" s="71"/>
+      <c r="E7" s="78"/>
+      <c r="F7" s="78"/>
+      <c r="G7" s="76"/>
+      <c r="H7" s="82"/>
+      <c r="I7" s="78"/>
     </row>
     <row r="8" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="86"/>
+      <c r="A8" s="135"/>
       <c r="B8" s="63">
         <v>3</v>
       </c>
@@ -1606,41 +1616,41 @@
       <c r="I8" s="3"/>
     </row>
     <row r="9" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="86"/>
-      <c r="B9" s="82">
+      <c r="A9" s="135"/>
+      <c r="B9" s="118">
         <v>4</v>
       </c>
-      <c r="C9" s="94" t="s">
+      <c r="C9" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="116" t="s">
+      <c r="D9" s="87" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="70"/>
-      <c r="F9" s="126"/>
+      <c r="E9" s="77"/>
+      <c r="F9" s="89"/>
       <c r="G9" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="H9" s="128"/>
-      <c r="I9" s="89" t="s">
+      <c r="H9" s="91"/>
+      <c r="I9" s="75" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="10" spans="1:9" s="35" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="86"/>
-      <c r="B10" s="93"/>
-      <c r="C10" s="95"/>
-      <c r="D10" s="118"/>
-      <c r="E10" s="71"/>
-      <c r="F10" s="127"/>
+      <c r="A10" s="135"/>
+      <c r="B10" s="119"/>
+      <c r="C10" s="74"/>
+      <c r="D10" s="88"/>
+      <c r="E10" s="78"/>
+      <c r="F10" s="90"/>
       <c r="G10" s="42" t="s">
         <v>110</v>
       </c>
-      <c r="H10" s="129"/>
-      <c r="I10" s="90"/>
+      <c r="H10" s="92"/>
+      <c r="I10" s="76"/>
     </row>
     <row r="11" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="86"/>
+      <c r="A11" s="135"/>
       <c r="B11" s="56">
         <v>5</v>
       </c>
@@ -1659,82 +1669,82 @@
       <c r="I11" s="37"/>
     </row>
     <row r="12" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="86"/>
-      <c r="B12" s="87">
+      <c r="A12" s="135"/>
+      <c r="B12" s="79">
         <v>6</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="89" t="s">
+      <c r="D12" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="133"/>
-      <c r="F12" s="133"/>
-      <c r="G12" s="70"/>
-      <c r="H12" s="89" t="s">
+      <c r="E12" s="83"/>
+      <c r="F12" s="83"/>
+      <c r="G12" s="77"/>
+      <c r="H12" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="70"/>
+      <c r="I12" s="77"/>
     </row>
     <row r="13" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="86"/>
-      <c r="B13" s="88"/>
+      <c r="A13" s="135"/>
+      <c r="B13" s="80"/>
       <c r="C13" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="90"/>
-      <c r="E13" s="134"/>
-      <c r="F13" s="134"/>
-      <c r="G13" s="71"/>
-      <c r="H13" s="90"/>
-      <c r="I13" s="71"/>
+      <c r="D13" s="76"/>
+      <c r="E13" s="84"/>
+      <c r="F13" s="84"/>
+      <c r="G13" s="78"/>
+      <c r="H13" s="76"/>
+      <c r="I13" s="78"/>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="86"/>
-      <c r="B14" s="82">
+      <c r="A14" s="135"/>
+      <c r="B14" s="118">
         <v>7</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="91" t="s">
+      <c r="D14" s="85" t="s">
         <v>108</v>
       </c>
-      <c r="E14" s="70"/>
-      <c r="F14" s="70"/>
-      <c r="G14" s="119" t="s">
+      <c r="E14" s="77"/>
+      <c r="F14" s="77"/>
+      <c r="G14" s="93" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="91"/>
-      <c r="I14" s="91"/>
+      <c r="H14" s="85"/>
+      <c r="I14" s="85"/>
     </row>
     <row r="15" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="86"/>
-      <c r="B15" s="93"/>
+      <c r="A15" s="135"/>
+      <c r="B15" s="119"/>
       <c r="C15" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="92"/>
-      <c r="E15" s="71"/>
-      <c r="F15" s="71"/>
-      <c r="G15" s="121"/>
-      <c r="H15" s="92"/>
-      <c r="I15" s="92"/>
+      <c r="D15" s="86"/>
+      <c r="E15" s="78"/>
+      <c r="F15" s="78"/>
+      <c r="G15" s="94"/>
+      <c r="H15" s="86"/>
+      <c r="I15" s="86"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="86"/>
-      <c r="B16" s="82">
+      <c r="A16" s="135"/>
+      <c r="B16" s="118">
         <v>8</v>
       </c>
-      <c r="C16" s="96"/>
+      <c r="C16" s="108"/>
       <c r="D16" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="99"/>
-      <c r="F16" s="70"/>
-      <c r="G16" s="119"/>
-      <c r="H16" s="96" t="s">
+      <c r="E16" s="120"/>
+      <c r="F16" s="77"/>
+      <c r="G16" s="93"/>
+      <c r="H16" s="108" t="s">
         <v>27</v>
       </c>
       <c r="I16" s="5" t="s">
@@ -1742,35 +1752,35 @@
       </c>
     </row>
     <row r="17" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A17" s="86"/>
-      <c r="B17" s="83"/>
-      <c r="C17" s="97"/>
+      <c r="A17" s="135"/>
+      <c r="B17" s="123"/>
+      <c r="C17" s="109"/>
       <c r="D17" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="100"/>
-      <c r="F17" s="79"/>
-      <c r="G17" s="120"/>
-      <c r="H17" s="97"/>
+      <c r="E17" s="121"/>
+      <c r="F17" s="95"/>
+      <c r="G17" s="111"/>
+      <c r="H17" s="109"/>
       <c r="I17" s="17" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="86"/>
-      <c r="B18" s="93"/>
-      <c r="C18" s="98"/>
+      <c r="A18" s="135"/>
+      <c r="B18" s="119"/>
+      <c r="C18" s="110"/>
       <c r="D18" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="101"/>
-      <c r="F18" s="71"/>
-      <c r="G18" s="121"/>
-      <c r="H18" s="98"/>
+      <c r="E18" s="122"/>
+      <c r="F18" s="78"/>
+      <c r="G18" s="94"/>
+      <c r="H18" s="110"/>
       <c r="I18" s="47"/>
     </row>
     <row r="19" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="86"/>
+      <c r="A19" s="135"/>
       <c r="B19" s="56">
         <v>9</v>
       </c>
@@ -1793,41 +1803,41 @@
       </c>
     </row>
     <row r="20" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A20" s="86"/>
-      <c r="B20" s="87">
+      <c r="A20" s="135"/>
+      <c r="B20" s="79">
         <v>10</v>
       </c>
       <c r="C20" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="70"/>
-      <c r="E20" s="89" t="s">
+      <c r="D20" s="77"/>
+      <c r="E20" s="75" t="s">
         <v>39</v>
       </c>
-      <c r="F20" s="89" t="s">
+      <c r="F20" s="75" t="s">
         <v>38</v>
       </c>
-      <c r="G20" s="70"/>
-      <c r="H20" s="103" t="s">
+      <c r="G20" s="77"/>
+      <c r="H20" s="100" t="s">
         <v>93</v>
       </c>
-      <c r="I20" s="70"/>
+      <c r="I20" s="77"/>
     </row>
     <row r="21" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="86"/>
-      <c r="B21" s="88"/>
+      <c r="A21" s="135"/>
+      <c r="B21" s="80"/>
       <c r="C21" s="54" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="71"/>
-      <c r="E21" s="90"/>
-      <c r="F21" s="90"/>
-      <c r="G21" s="71"/>
-      <c r="H21" s="104"/>
-      <c r="I21" s="71"/>
+      <c r="D21" s="78"/>
+      <c r="E21" s="76"/>
+      <c r="F21" s="76"/>
+      <c r="G21" s="78"/>
+      <c r="H21" s="101"/>
+      <c r="I21" s="78"/>
     </row>
     <row r="22" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="86"/>
+      <c r="A22" s="135"/>
       <c r="B22" s="56">
         <v>11</v>
       </c>
@@ -1844,7 +1854,7 @@
       <c r="I22" s="4"/>
     </row>
     <row r="23" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="86"/>
+      <c r="A23" s="135"/>
       <c r="B23" s="62">
         <v>12</v>
       </c>
@@ -1861,8 +1871,8 @@
       <c r="I23" s="46"/>
     </row>
     <row r="24" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A24" s="86"/>
-      <c r="B24" s="87">
+      <c r="A24" s="135"/>
+      <c r="B24" s="79">
         <v>13</v>
       </c>
       <c r="C24" s="21" t="s">
@@ -1871,84 +1881,84 @@
       <c r="D24" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="E24" s="103"/>
-      <c r="F24" s="109"/>
+      <c r="E24" s="100"/>
+      <c r="F24" s="113"/>
       <c r="G24" s="36" t="s">
         <v>48</v>
       </c>
       <c r="H24" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="I24" s="70"/>
+      <c r="I24" s="77"/>
     </row>
     <row r="25" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A25" s="86"/>
-      <c r="B25" s="102"/>
+      <c r="A25" s="135"/>
+      <c r="B25" s="103"/>
       <c r="C25" s="9" t="s">
         <v>42</v>
       </c>
       <c r="D25" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="E25" s="111"/>
-      <c r="F25" s="123"/>
+      <c r="E25" s="116"/>
+      <c r="F25" s="114"/>
       <c r="G25" s="19" t="s">
         <v>45</v>
       </c>
       <c r="H25" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="I25" s="79"/>
+      <c r="I25" s="95"/>
     </row>
     <row r="26" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="86"/>
-      <c r="B26" s="88"/>
+      <c r="A26" s="135"/>
+      <c r="B26" s="80"/>
       <c r="C26" s="47"/>
       <c r="D26" s="49"/>
-      <c r="E26" s="104"/>
-      <c r="F26" s="110"/>
+      <c r="E26" s="101"/>
+      <c r="F26" s="115"/>
       <c r="G26" s="20" t="s">
         <v>44</v>
       </c>
       <c r="H26" s="42"/>
-      <c r="I26" s="71"/>
+      <c r="I26" s="78"/>
     </row>
     <row r="27" spans="1:9" ht="21" x14ac:dyDescent="0.3">
-      <c r="A27" s="86"/>
-      <c r="B27" s="87">
+      <c r="A27" s="135"/>
+      <c r="B27" s="79">
         <v>14</v>
       </c>
-      <c r="C27" s="107"/>
-      <c r="D27" s="109"/>
+      <c r="C27" s="96"/>
+      <c r="D27" s="113"/>
       <c r="E27" s="29" t="s">
         <v>53</v>
       </c>
       <c r="F27" s="51" t="s">
         <v>52</v>
       </c>
-      <c r="G27" s="107"/>
-      <c r="H27" s="124" t="s">
+      <c r="G27" s="96"/>
+      <c r="H27" s="98" t="s">
         <v>95</v>
       </c>
-      <c r="I27" s="70"/>
+      <c r="I27" s="77"/>
     </row>
     <row r="28" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="86"/>
-      <c r="B28" s="88"/>
-      <c r="C28" s="108"/>
-      <c r="D28" s="110"/>
+      <c r="A28" s="135"/>
+      <c r="B28" s="80"/>
+      <c r="C28" s="97"/>
+      <c r="D28" s="115"/>
       <c r="E28" s="53" t="s">
         <v>55</v>
       </c>
       <c r="F28" s="52" t="s">
         <v>54</v>
       </c>
-      <c r="G28" s="108"/>
-      <c r="H28" s="125"/>
-      <c r="I28" s="71"/>
+      <c r="G28" s="97"/>
+      <c r="H28" s="99"/>
+      <c r="I28" s="78"/>
     </row>
     <row r="29" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="86"/>
+      <c r="A29" s="135"/>
       <c r="B29" s="66">
         <v>15</v>
       </c>
@@ -1969,254 +1979,307 @@
       <c r="I29" s="2"/>
     </row>
     <row r="30" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="86"/>
-      <c r="B30" s="87">
+      <c r="A30" s="135"/>
+      <c r="B30" s="79">
         <v>16</v>
       </c>
       <c r="C30" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="D30" s="103" t="s">
+      <c r="D30" s="100" t="s">
         <v>58</v>
       </c>
-      <c r="E30" s="105"/>
-      <c r="F30" s="70"/>
-      <c r="G30" s="70"/>
-      <c r="H30" s="89" t="s">
+      <c r="E30" s="124"/>
+      <c r="F30" s="77"/>
+      <c r="G30" s="77"/>
+      <c r="H30" s="75" t="s">
         <v>61</v>
       </c>
-      <c r="I30" s="91" t="s">
+      <c r="I30" s="85" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="86"/>
-      <c r="B31" s="88"/>
+      <c r="A31" s="135"/>
+      <c r="B31" s="80"/>
       <c r="C31" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="D31" s="104"/>
-      <c r="E31" s="106"/>
-      <c r="F31" s="71"/>
-      <c r="G31" s="71"/>
-      <c r="H31" s="90"/>
-      <c r="I31" s="92"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A32" s="86"/>
-      <c r="B32" s="82">
+      <c r="D31" s="101"/>
+      <c r="E31" s="125"/>
+      <c r="F31" s="78"/>
+      <c r="G31" s="78"/>
+      <c r="H31" s="76"/>
+      <c r="I31" s="86"/>
+    </row>
+    <row r="32" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="A32" s="135"/>
+      <c r="B32" s="118">
         <v>17</v>
       </c>
-      <c r="C32" s="5"/>
+      <c r="C32" s="17" t="s">
+        <v>104</v>
+      </c>
       <c r="D32" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="E32" s="70"/>
-      <c r="F32" s="70"/>
-      <c r="G32" s="80" t="s">
+      <c r="E32" s="77"/>
+      <c r="F32" s="77"/>
+      <c r="G32" s="132" t="s">
         <v>68</v>
       </c>
-      <c r="H32" s="91" t="s">
+      <c r="H32" s="85" t="s">
         <v>64</v>
       </c>
       <c r="I32" s="7" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A33" s="86"/>
-      <c r="B33" s="83"/>
-      <c r="C33" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="D33" s="39" t="s">
-        <v>100</v>
-      </c>
-      <c r="E33" s="79"/>
-      <c r="F33" s="79"/>
-      <c r="G33" s="81"/>
-      <c r="H33" s="122"/>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" s="135"/>
+      <c r="B33" s="123"/>
+      <c r="C33" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="D33" s="72" t="s">
+        <v>74</v>
+      </c>
+      <c r="E33" s="95"/>
+      <c r="F33" s="95"/>
+      <c r="G33" s="133"/>
+      <c r="H33" s="112"/>
       <c r="I33" s="41" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="86"/>
-      <c r="B34" s="83"/>
-      <c r="C34" s="34" t="s">
-        <v>62</v>
-      </c>
-      <c r="D34" s="85" t="s">
-        <v>74</v>
-      </c>
-      <c r="E34" s="79"/>
-      <c r="F34" s="79"/>
-      <c r="G34" s="81"/>
-      <c r="H34" s="122"/>
-      <c r="I34" s="115"/>
-    </row>
-    <row r="35" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A35" s="86"/>
-      <c r="B35" s="83"/>
-      <c r="C35" s="9" t="s">
+    <row r="34" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A34" s="135"/>
+      <c r="B34" s="123"/>
+      <c r="C34" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D35" s="85"/>
-      <c r="E35" s="79"/>
-      <c r="F35" s="79"/>
-      <c r="G35" s="81"/>
-      <c r="H35" s="122"/>
-      <c r="I35" s="115"/>
+      <c r="D34" s="69"/>
+      <c r="E34" s="95"/>
+      <c r="F34" s="95"/>
+      <c r="G34" s="133"/>
+      <c r="H34" s="112"/>
+      <c r="I34" s="71"/>
+    </row>
+    <row r="35" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="A35" s="135"/>
+      <c r="B35" s="79">
+        <v>18</v>
+      </c>
+      <c r="C35" s="104"/>
+      <c r="D35" s="70" t="s">
+        <v>105</v>
+      </c>
+      <c r="E35" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="F35" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="G35" s="77"/>
+      <c r="H35" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="I35" s="87" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="36" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A36" s="86"/>
-      <c r="B36" s="87">
-        <v>18</v>
-      </c>
-      <c r="C36" s="112"/>
-      <c r="D36" s="94" t="s">
-        <v>105</v>
-      </c>
-      <c r="E36" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="F36" s="18" t="s">
-        <v>107</v>
-      </c>
-      <c r="G36" s="70"/>
-      <c r="H36" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="I36" s="116" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A37" s="86"/>
-      <c r="B37" s="102"/>
-      <c r="C37" s="113"/>
-      <c r="D37" s="130"/>
-      <c r="E37" s="17" t="s">
+      <c r="A36" s="135"/>
+      <c r="B36" s="103"/>
+      <c r="C36" s="105"/>
+      <c r="D36" s="39" t="s">
+        <v>100</v>
+      </c>
+      <c r="E36" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="F37" s="40" t="s">
+      <c r="F36" s="40" t="s">
         <v>72</v>
       </c>
-      <c r="G37" s="79"/>
-      <c r="H37" s="6" t="s">
+      <c r="G36" s="95"/>
+      <c r="H36" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I37" s="117"/>
-    </row>
-    <row r="38" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A38" s="86"/>
-      <c r="B38" s="88"/>
-      <c r="C38" s="114"/>
-      <c r="D38" s="95"/>
-      <c r="E38" s="20" t="s">
+      <c r="I36" s="107"/>
+    </row>
+    <row r="37" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A37" s="135"/>
+      <c r="B37" s="80"/>
+      <c r="C37" s="106"/>
+      <c r="D37" s="136"/>
+      <c r="E37" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="F38" s="12" t="s">
+      <c r="F37" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="G38" s="71"/>
-      <c r="H38" s="33"/>
-      <c r="I38" s="118"/>
-    </row>
-    <row r="39" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A39" s="86"/>
-      <c r="B39" s="63">
+      <c r="G37" s="78"/>
+      <c r="H37" s="33"/>
+      <c r="I37" s="88"/>
+    </row>
+    <row r="38" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="135"/>
+      <c r="B38" s="63">
         <v>20</v>
       </c>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="13" t="s">
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="I39" s="10" t="s">
+      <c r="I38" s="10" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="69"/>
-      <c r="B40" s="77" t="s">
+    <row r="39" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A39" s="117"/>
+      <c r="B39" s="102" t="s">
         <v>86</v>
       </c>
-      <c r="C40" s="77"/>
-      <c r="D40" s="77"/>
-      <c r="E40" s="77"/>
-      <c r="F40" s="77"/>
-      <c r="G40" s="77"/>
-      <c r="H40" s="77"/>
-      <c r="I40" s="78"/>
-    </row>
-    <row r="41" spans="1:9" s="14" customFormat="1" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="69"/>
-      <c r="B41" s="16"/>
-      <c r="C41" s="15">
-        <f>COUNTIF(C4:C39, "&lt;&gt;")</f>
+      <c r="C39" s="102"/>
+      <c r="D39" s="102"/>
+      <c r="E39" s="102"/>
+      <c r="F39" s="102"/>
+      <c r="G39" s="102"/>
+      <c r="H39" s="102"/>
+      <c r="I39" s="131"/>
+    </row>
+    <row r="40" spans="1:9" s="14" customFormat="1" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A40" s="117"/>
+      <c r="B40" s="16"/>
+      <c r="C40" s="15">
+        <f>COUNTIF(C4:C38, "&lt;&gt;")</f>
         <v>20</v>
       </c>
-      <c r="D41" s="15">
-        <f>COUNTIF(D4:D39, "&lt;&gt;")</f>
+      <c r="D40" s="15">
+        <f>COUNTIF(D4:D38, "&lt;&gt;")</f>
         <v>20</v>
       </c>
-      <c r="E41" s="15">
-        <f t="shared" ref="E41:I41" si="0">COUNTIF(E4:E39, "&lt;&gt;")</f>
+      <c r="E40" s="15">
+        <f t="shared" ref="E40:I40" si="0">COUNTIF(E4:E38, "&lt;&gt;")</f>
         <v>9</v>
       </c>
-      <c r="F41" s="15">
+      <c r="F40" s="15">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="G41" s="15">
+      <c r="G40" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="H41" s="15">
+      <c r="H40" s="15">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="I41" s="15">
+      <c r="I40" s="15">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="69"/>
-      <c r="B42" s="77" t="str">
-        <f>SUM(C41:I41) &amp; " Total Races (Prior to Breeders' Cup Weekend)"</f>
+    <row r="41" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A41" s="117"/>
+      <c r="B41" s="102" t="str">
+        <f>SUM(C40:I40) &amp; " Total Races (Prior to Breeders' Cup Weekend)"</f>
         <v>94 Total Races (Prior to Breeders' Cup Weekend)</v>
       </c>
-      <c r="C42" s="77"/>
-      <c r="D42" s="77"/>
-      <c r="E42" s="77"/>
-      <c r="F42" s="77"/>
-      <c r="G42" s="77"/>
-      <c r="H42" s="77"/>
-      <c r="I42" s="77"/>
-    </row>
-    <row r="43" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A43" s="69"/>
-      <c r="B43" s="72" t="s">
+      <c r="C41" s="102"/>
+      <c r="D41" s="102"/>
+      <c r="E41" s="102"/>
+      <c r="F41" s="102"/>
+      <c r="G41" s="102"/>
+      <c r="H41" s="102"/>
+      <c r="I41" s="102"/>
+    </row>
+    <row r="42" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A42" s="117"/>
+      <c r="B42" s="126" t="s">
         <v>84</v>
       </c>
-      <c r="C43" s="72"/>
-      <c r="D43" s="72"/>
-      <c r="E43" s="73"/>
-      <c r="F43" s="74" t="s">
+      <c r="C42" s="126"/>
+      <c r="D42" s="126"/>
+      <c r="E42" s="127"/>
+      <c r="F42" s="128" t="s">
         <v>85</v>
       </c>
-      <c r="G43" s="75"/>
-      <c r="H43" s="75"/>
-      <c r="I43" s="76"/>
+      <c r="G42" s="129"/>
+      <c r="H42" s="129"/>
+      <c r="I42" s="130"/>
     </row>
   </sheetData>
-  <mergeCells count="83">
-    <mergeCell ref="D36:D38"/>
+  <mergeCells count="80">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="F42:I42"/>
+    <mergeCell ref="B39:I39"/>
+    <mergeCell ref="E32:E34"/>
+    <mergeCell ref="F32:F34"/>
+    <mergeCell ref="G32:G34"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="C1:I1"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="A2:A38"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="F30:F31"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="A39:A42"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="I30:I31"/>
+    <mergeCell ref="G30:G31"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="I12:I13"/>
+    <mergeCell ref="H20:H21"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="G35:G37"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="C35:C37"/>
+    <mergeCell ref="I35:I37"/>
+    <mergeCell ref="H16:H18"/>
+    <mergeCell ref="G16:G18"/>
+    <mergeCell ref="F16:F18"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="F24:F26"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="I24:I26"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="H27:H28"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="H9:H10"/>
     <mergeCell ref="H30:H31"/>
     <mergeCell ref="I20:I21"/>
     <mergeCell ref="B6:B7"/>
@@ -2232,73 +2295,6 @@
     <mergeCell ref="F12:F13"/>
     <mergeCell ref="G12:G13"/>
     <mergeCell ref="D14:D15"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="I24:I26"/>
-    <mergeCell ref="G27:G28"/>
-    <mergeCell ref="H27:H28"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="H12:H13"/>
-    <mergeCell ref="I12:I13"/>
-    <mergeCell ref="H20:H21"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="B42:I42"/>
-    <mergeCell ref="G36:G38"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="C36:C38"/>
-    <mergeCell ref="I34:I35"/>
-    <mergeCell ref="I36:I38"/>
-    <mergeCell ref="H16:H18"/>
-    <mergeCell ref="G16:G18"/>
-    <mergeCell ref="F16:F18"/>
-    <mergeCell ref="H32:H35"/>
-    <mergeCell ref="F24:F26"/>
-    <mergeCell ref="I30:I31"/>
-    <mergeCell ref="G30:G31"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="F30:F31"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="A40:A43"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="E16:E18"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="B43:E43"/>
-    <mergeCell ref="F43:I43"/>
-    <mergeCell ref="B40:I40"/>
-    <mergeCell ref="E32:E35"/>
-    <mergeCell ref="F32:F35"/>
-    <mergeCell ref="G32:G35"/>
-    <mergeCell ref="B32:B35"/>
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="A2:A39"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="D20:D21"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="51" fitToHeight="10" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
GRCW-1096; RTTR153 Prep Race Results
</commit_message>
<xml_diff>
--- a/pdf/RTTBC26-Schedule-by-Division.xlsx
+++ b/pdf/RTTBC26-Schedule-by-Division.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/299f8723705ec823/Webmaster/gallop-racing/pdf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1622" documentId="8_{DAECCBE5-FF72-4188-B2F1-1541968A3FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{750E098A-DDA0-4D5B-9FEF-95D99D67400B}"/>
+  <xr:revisionPtr revIDLastSave="1624" documentId="8_{DAECCBE5-FF72-4188-B2F1-1541968A3FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5711646A-2FC7-4D27-A622-D341ECBCF267}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{EAD27B02-19FE-4D48-9014-ED6E24DB84F0}"/>
   </bookViews>
@@ -248,9 +248,6 @@
     <t>Zenyatta S.-G2</t>
   </si>
   <si>
-    <t>S. K. Ogden Phoenix S.-G2</t>
-  </si>
-  <si>
     <t>Champagne S.-G1</t>
   </si>
   <si>
@@ -266,9 +263,6 @@
     <t>T'bred Club of America S.-G2</t>
   </si>
   <si>
-    <t>Lexus Raven Run S.-G2</t>
-  </si>
-  <si>
     <t>BC JUVENILE-G1</t>
   </si>
   <si>
@@ -372,6 +366,12 @@
   </si>
   <si>
     <t>Bango S.-G3</t>
+  </si>
+  <si>
+    <t>Raven Run S.-G2</t>
+  </si>
+  <si>
+    <t>Phoenix S.-G2</t>
   </si>
 </sst>
 </file>
@@ -723,7 +723,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="136">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -935,17 +935,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -953,169 +944,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1124,8 +986,143 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1464,47 +1461,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="117"/>
-      <c r="B1" s="117"/>
-      <c r="C1" s="134" t="s">
-        <v>87</v>
-      </c>
-      <c r="D1" s="134"/>
-      <c r="E1" s="134"/>
-      <c r="F1" s="134"/>
-      <c r="G1" s="134"/>
-      <c r="H1" s="134"/>
-      <c r="I1" s="134"/>
+      <c r="A1" s="73"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="88" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
     </row>
     <row r="2" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A2" s="135" t="s">
-        <v>88</v>
+      <c r="A2" s="89" t="s">
+        <v>86</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="24" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D2" s="24" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E2" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="F2" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="G2" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="H2" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="I2" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="G2" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="H2" s="24" t="s">
-        <v>79</v>
-      </c>
-      <c r="I2" s="24" t="s">
-        <v>80</v>
-      </c>
     </row>
     <row r="3" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="135"/>
+      <c r="A3" s="89"/>
       <c r="B3" s="27"/>
       <c r="C3" s="25" t="s">
         <v>5</v>
@@ -1529,8 +1526,8 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A4" s="135"/>
-      <c r="B4" s="118">
+      <c r="A4" s="89"/>
+      <c r="B4" s="86">
         <v>1</v>
       </c>
       <c r="C4" s="21" t="s">
@@ -1539,67 +1536,67 @@
       <c r="D4" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="77"/>
-      <c r="F4" s="77"/>
-      <c r="G4" s="73" t="s">
+      <c r="E4" s="74"/>
+      <c r="F4" s="74"/>
+      <c r="G4" s="95" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="85" t="s">
-        <v>89</v>
+      <c r="H4" s="92" t="s">
+        <v>87</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="135"/>
-      <c r="B5" s="119"/>
+      <c r="A5" s="89"/>
+      <c r="B5" s="94"/>
       <c r="C5" s="11" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="64" t="s">
-        <v>103</v>
-      </c>
-      <c r="E5" s="78"/>
-      <c r="F5" s="78"/>
-      <c r="G5" s="74"/>
-      <c r="H5" s="86"/>
+        <v>101</v>
+      </c>
+      <c r="E5" s="75"/>
+      <c r="F5" s="75"/>
+      <c r="G5" s="96"/>
+      <c r="H5" s="93"/>
       <c r="I5" s="65" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="135"/>
-      <c r="B6" s="79">
+      <c r="A6" s="89"/>
+      <c r="B6" s="90">
         <v>2</v>
       </c>
-      <c r="C6" s="77"/>
+      <c r="C6" s="74"/>
       <c r="D6" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="77"/>
-      <c r="F6" s="77"/>
-      <c r="G6" s="75" t="s">
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
+      <c r="G6" s="103" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="81"/>
-      <c r="I6" s="77"/>
+      <c r="H6" s="132"/>
+      <c r="I6" s="74"/>
     </row>
     <row r="7" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="135"/>
-      <c r="B7" s="80"/>
-      <c r="C7" s="78"/>
+      <c r="A7" s="89"/>
+      <c r="B7" s="91"/>
+      <c r="C7" s="75"/>
       <c r="D7" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="E7" s="78"/>
-      <c r="F7" s="78"/>
-      <c r="G7" s="76"/>
-      <c r="H7" s="82"/>
-      <c r="I7" s="78"/>
+        <v>97</v>
+      </c>
+      <c r="E7" s="75"/>
+      <c r="F7" s="75"/>
+      <c r="G7" s="104"/>
+      <c r="H7" s="133"/>
+      <c r="I7" s="75"/>
     </row>
     <row r="8" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="135"/>
+      <c r="A8" s="89"/>
       <c r="B8" s="63">
         <v>3</v>
       </c>
@@ -1611,46 +1608,46 @@
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="38" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="I8" s="3"/>
     </row>
     <row r="9" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="135"/>
-      <c r="B9" s="118">
+      <c r="A9" s="89"/>
+      <c r="B9" s="86">
         <v>4</v>
       </c>
-      <c r="C9" s="73" t="s">
+      <c r="C9" s="95" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="87" t="s">
+      <c r="D9" s="118" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="77"/>
-      <c r="F9" s="89"/>
+      <c r="E9" s="74"/>
+      <c r="F9" s="128"/>
       <c r="G9" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="H9" s="130"/>
+      <c r="I9" s="103" t="s">
         <v>109</v>
       </c>
-      <c r="H9" s="91"/>
-      <c r="I9" s="75" t="s">
-        <v>111</v>
-      </c>
     </row>
     <row r="10" spans="1:9" s="35" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="135"/>
-      <c r="B10" s="119"/>
-      <c r="C10" s="74"/>
-      <c r="D10" s="88"/>
-      <c r="E10" s="78"/>
-      <c r="F10" s="90"/>
+      <c r="A10" s="89"/>
+      <c r="B10" s="94"/>
+      <c r="C10" s="96"/>
+      <c r="D10" s="120"/>
+      <c r="E10" s="75"/>
+      <c r="F10" s="129"/>
       <c r="G10" s="42" t="s">
-        <v>110</v>
-      </c>
-      <c r="H10" s="92"/>
-      <c r="I10" s="76"/>
+        <v>108</v>
+      </c>
+      <c r="H10" s="131"/>
+      <c r="I10" s="104"/>
     </row>
     <row r="11" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="135"/>
+      <c r="A11" s="89"/>
       <c r="B11" s="56">
         <v>5</v>
       </c>
@@ -1669,118 +1666,118 @@
       <c r="I11" s="37"/>
     </row>
     <row r="12" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="135"/>
-      <c r="B12" s="79">
+      <c r="A12" s="89"/>
+      <c r="B12" s="90">
         <v>6</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="75" t="s">
+      <c r="D12" s="103" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="83"/>
-      <c r="F12" s="83"/>
-      <c r="G12" s="77"/>
-      <c r="H12" s="75" t="s">
+      <c r="E12" s="134"/>
+      <c r="F12" s="134"/>
+      <c r="G12" s="74"/>
+      <c r="H12" s="103" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="77"/>
+      <c r="I12" s="74"/>
     </row>
     <row r="13" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="135"/>
-      <c r="B13" s="80"/>
+      <c r="A13" s="89"/>
+      <c r="B13" s="91"/>
       <c r="C13" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="76"/>
-      <c r="E13" s="84"/>
-      <c r="F13" s="84"/>
-      <c r="G13" s="78"/>
-      <c r="H13" s="76"/>
-      <c r="I13" s="78"/>
+      <c r="D13" s="104"/>
+      <c r="E13" s="135"/>
+      <c r="F13" s="135"/>
+      <c r="G13" s="75"/>
+      <c r="H13" s="104"/>
+      <c r="I13" s="75"/>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="135"/>
-      <c r="B14" s="118">
+      <c r="A14" s="89"/>
+      <c r="B14" s="86">
         <v>7</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="85" t="s">
-        <v>108</v>
-      </c>
-      <c r="E14" s="77"/>
-      <c r="F14" s="77"/>
-      <c r="G14" s="93" t="s">
+      <c r="D14" s="92" t="s">
+        <v>106</v>
+      </c>
+      <c r="E14" s="74"/>
+      <c r="F14" s="74"/>
+      <c r="G14" s="121" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="85"/>
-      <c r="I14" s="85"/>
+      <c r="H14" s="92"/>
+      <c r="I14" s="92"/>
     </row>
     <row r="15" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="135"/>
-      <c r="B15" s="119"/>
+      <c r="A15" s="89"/>
+      <c r="B15" s="94"/>
       <c r="C15" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="86"/>
-      <c r="E15" s="78"/>
-      <c r="F15" s="78"/>
-      <c r="G15" s="94"/>
-      <c r="H15" s="86"/>
-      <c r="I15" s="86"/>
+      <c r="D15" s="93"/>
+      <c r="E15" s="75"/>
+      <c r="F15" s="75"/>
+      <c r="G15" s="123"/>
+      <c r="H15" s="93"/>
+      <c r="I15" s="93"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="135"/>
-      <c r="B16" s="118">
+      <c r="A16" s="89"/>
+      <c r="B16" s="86">
         <v>8</v>
       </c>
-      <c r="C16" s="108"/>
+      <c r="C16" s="97"/>
       <c r="D16" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="120"/>
-      <c r="F16" s="77"/>
-      <c r="G16" s="93"/>
-      <c r="H16" s="108" t="s">
+      <c r="E16" s="100"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="121"/>
+      <c r="H16" s="97" t="s">
         <v>27</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A17" s="135"/>
-      <c r="B17" s="123"/>
-      <c r="C17" s="109"/>
+      <c r="A17" s="89"/>
+      <c r="B17" s="87"/>
+      <c r="C17" s="98"/>
       <c r="D17" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="121"/>
-      <c r="F17" s="95"/>
-      <c r="G17" s="111"/>
-      <c r="H17" s="109"/>
+      <c r="E17" s="101"/>
+      <c r="F17" s="83"/>
+      <c r="G17" s="122"/>
+      <c r="H17" s="98"/>
       <c r="I17" s="17" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="135"/>
-      <c r="B18" s="119"/>
-      <c r="C18" s="110"/>
+      <c r="A18" s="89"/>
+      <c r="B18" s="94"/>
+      <c r="C18" s="99"/>
       <c r="D18" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="122"/>
-      <c r="F18" s="78"/>
-      <c r="G18" s="94"/>
-      <c r="H18" s="110"/>
+      <c r="E18" s="102"/>
+      <c r="F18" s="75"/>
+      <c r="G18" s="123"/>
+      <c r="H18" s="99"/>
       <c r="I18" s="47"/>
     </row>
     <row r="19" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="135"/>
+      <c r="A19" s="89"/>
       <c r="B19" s="56">
         <v>9</v>
       </c>
@@ -1803,41 +1800,41 @@
       </c>
     </row>
     <row r="20" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A20" s="135"/>
-      <c r="B20" s="79">
+      <c r="A20" s="89"/>
+      <c r="B20" s="90">
         <v>10</v>
       </c>
       <c r="C20" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="77"/>
-      <c r="E20" s="75" t="s">
+      <c r="D20" s="74"/>
+      <c r="E20" s="103" t="s">
         <v>39</v>
       </c>
-      <c r="F20" s="75" t="s">
+      <c r="F20" s="103" t="s">
         <v>38</v>
       </c>
-      <c r="G20" s="77"/>
-      <c r="H20" s="100" t="s">
-        <v>93</v>
-      </c>
-      <c r="I20" s="77"/>
+      <c r="G20" s="74"/>
+      <c r="H20" s="106" t="s">
+        <v>91</v>
+      </c>
+      <c r="I20" s="74"/>
     </row>
     <row r="21" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="135"/>
-      <c r="B21" s="80"/>
+      <c r="A21" s="89"/>
+      <c r="B21" s="91"/>
       <c r="C21" s="54" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="78"/>
-      <c r="E21" s="76"/>
-      <c r="F21" s="76"/>
-      <c r="G21" s="78"/>
-      <c r="H21" s="101"/>
-      <c r="I21" s="78"/>
+      <c r="D21" s="75"/>
+      <c r="E21" s="104"/>
+      <c r="F21" s="104"/>
+      <c r="G21" s="75"/>
+      <c r="H21" s="107"/>
+      <c r="I21" s="75"/>
     </row>
     <row r="22" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="135"/>
+      <c r="A22" s="89"/>
       <c r="B22" s="56">
         <v>11</v>
       </c>
@@ -1854,7 +1851,7 @@
       <c r="I22" s="4"/>
     </row>
     <row r="23" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="135"/>
+      <c r="A23" s="89"/>
       <c r="B23" s="62">
         <v>12</v>
       </c>
@@ -1871,100 +1868,100 @@
       <c r="I23" s="46"/>
     </row>
     <row r="24" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A24" s="135"/>
-      <c r="B24" s="79">
+      <c r="A24" s="89"/>
+      <c r="B24" s="90">
         <v>13</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D24" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="E24" s="100"/>
-      <c r="F24" s="113"/>
+      <c r="E24" s="106"/>
+      <c r="F24" s="112"/>
       <c r="G24" s="36" t="s">
         <v>48</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="I24" s="77"/>
+        <v>94</v>
+      </c>
+      <c r="I24" s="74"/>
     </row>
     <row r="25" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A25" s="135"/>
-      <c r="B25" s="103"/>
+      <c r="A25" s="89"/>
+      <c r="B25" s="105"/>
       <c r="C25" s="9" t="s">
         <v>42</v>
       </c>
       <c r="D25" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="E25" s="116"/>
-      <c r="F25" s="114"/>
+      <c r="E25" s="114"/>
+      <c r="F25" s="125"/>
       <c r="G25" s="19" t="s">
         <v>45</v>
       </c>
       <c r="H25" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="I25" s="95"/>
+      <c r="I25" s="83"/>
     </row>
     <row r="26" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="135"/>
-      <c r="B26" s="80"/>
+      <c r="A26" s="89"/>
+      <c r="B26" s="91"/>
       <c r="C26" s="47"/>
       <c r="D26" s="49"/>
-      <c r="E26" s="101"/>
-      <c r="F26" s="115"/>
+      <c r="E26" s="107"/>
+      <c r="F26" s="113"/>
       <c r="G26" s="20" t="s">
         <v>44</v>
       </c>
       <c r="H26" s="42"/>
-      <c r="I26" s="78"/>
+      <c r="I26" s="75"/>
     </row>
     <row r="27" spans="1:9" ht="21" x14ac:dyDescent="0.3">
-      <c r="A27" s="135"/>
-      <c r="B27" s="79">
+      <c r="A27" s="89"/>
+      <c r="B27" s="90">
         <v>14</v>
       </c>
-      <c r="C27" s="96"/>
-      <c r="D27" s="113"/>
+      <c r="C27" s="110"/>
+      <c r="D27" s="112"/>
       <c r="E27" s="29" t="s">
         <v>53</v>
       </c>
       <c r="F27" s="51" t="s">
         <v>52</v>
       </c>
-      <c r="G27" s="96"/>
-      <c r="H27" s="98" t="s">
-        <v>95</v>
-      </c>
-      <c r="I27" s="77"/>
+      <c r="G27" s="110"/>
+      <c r="H27" s="126" t="s">
+        <v>93</v>
+      </c>
+      <c r="I27" s="74"/>
     </row>
     <row r="28" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="135"/>
-      <c r="B28" s="80"/>
-      <c r="C28" s="97"/>
-      <c r="D28" s="115"/>
+      <c r="A28" s="89"/>
+      <c r="B28" s="91"/>
+      <c r="C28" s="111"/>
+      <c r="D28" s="113"/>
       <c r="E28" s="53" t="s">
         <v>55</v>
       </c>
       <c r="F28" s="52" t="s">
         <v>54</v>
       </c>
-      <c r="G28" s="97"/>
-      <c r="H28" s="99"/>
-      <c r="I28" s="78"/>
+      <c r="G28" s="111"/>
+      <c r="H28" s="127"/>
+      <c r="I28" s="75"/>
     </row>
     <row r="29" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="135"/>
+      <c r="A29" s="89"/>
       <c r="B29" s="66">
         <v>15</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E29" s="31" t="s">
         <v>56</v>
@@ -1974,61 +1971,61 @@
       </c>
       <c r="G29" s="2"/>
       <c r="H29" s="68" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I29" s="2"/>
     </row>
     <row r="30" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="135"/>
-      <c r="B30" s="79">
+      <c r="A30" s="89"/>
+      <c r="B30" s="90">
         <v>16</v>
       </c>
       <c r="C30" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="D30" s="100" t="s">
+      <c r="D30" s="106" t="s">
         <v>58</v>
       </c>
-      <c r="E30" s="124"/>
-      <c r="F30" s="77"/>
-      <c r="G30" s="77"/>
-      <c r="H30" s="75" t="s">
+      <c r="E30" s="108"/>
+      <c r="F30" s="74"/>
+      <c r="G30" s="74"/>
+      <c r="H30" s="103" t="s">
         <v>61</v>
       </c>
-      <c r="I30" s="85" t="s">
+      <c r="I30" s="92" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="135"/>
-      <c r="B31" s="80"/>
+      <c r="A31" s="89"/>
+      <c r="B31" s="91"/>
       <c r="C31" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="D31" s="101"/>
-      <c r="E31" s="125"/>
-      <c r="F31" s="78"/>
-      <c r="G31" s="78"/>
-      <c r="H31" s="76"/>
-      <c r="I31" s="86"/>
+      <c r="D31" s="107"/>
+      <c r="E31" s="109"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="104"/>
+      <c r="I31" s="93"/>
     </row>
     <row r="32" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A32" s="135"/>
-      <c r="B32" s="118">
+      <c r="A32" s="89"/>
+      <c r="B32" s="86">
         <v>17</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D32" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="E32" s="77"/>
-      <c r="F32" s="77"/>
-      <c r="G32" s="132" t="s">
+      <c r="E32" s="74"/>
+      <c r="F32" s="74"/>
+      <c r="G32" s="84" t="s">
         <v>68</v>
       </c>
-      <c r="H32" s="85" t="s">
+      <c r="H32" s="92" t="s">
         <v>64</v>
       </c>
       <c r="I32" s="7" t="s">
@@ -2036,94 +2033,94 @@
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" s="135"/>
-      <c r="B33" s="123"/>
+      <c r="A33" s="89"/>
+      <c r="B33" s="87"/>
       <c r="C33" s="34" t="s">
         <v>62</v>
       </c>
       <c r="D33" s="72" t="s">
-        <v>74</v>
-      </c>
-      <c r="E33" s="95"/>
-      <c r="F33" s="95"/>
-      <c r="G33" s="133"/>
-      <c r="H33" s="112"/>
+        <v>73</v>
+      </c>
+      <c r="E33" s="83"/>
+      <c r="F33" s="83"/>
+      <c r="G33" s="85"/>
+      <c r="H33" s="124"/>
       <c r="I33" s="41" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="135"/>
-      <c r="B34" s="123"/>
+      <c r="A34" s="89"/>
+      <c r="B34" s="87"/>
       <c r="C34" s="9" t="s">
         <v>67</v>
       </c>
       <c r="D34" s="69"/>
-      <c r="E34" s="95"/>
-      <c r="F34" s="95"/>
-      <c r="G34" s="133"/>
-      <c r="H34" s="112"/>
+      <c r="E34" s="83"/>
+      <c r="F34" s="83"/>
+      <c r="G34" s="85"/>
+      <c r="H34" s="124"/>
       <c r="I34" s="71"/>
     </row>
     <row r="35" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A35" s="135"/>
-      <c r="B35" s="79">
+      <c r="A35" s="89"/>
+      <c r="B35" s="90">
         <v>18</v>
       </c>
-      <c r="C35" s="104"/>
+      <c r="C35" s="115"/>
       <c r="D35" s="70" t="s">
+        <v>103</v>
+      </c>
+      <c r="E35" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="F35" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="E35" s="18" t="s">
+      <c r="G35" s="74"/>
+      <c r="H35" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="I35" s="118" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="A36" s="89"/>
+      <c r="B36" s="105"/>
+      <c r="C36" s="116"/>
+      <c r="D36" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="F36" s="40" t="s">
         <v>71</v>
       </c>
-      <c r="F35" s="18" t="s">
-        <v>107</v>
-      </c>
-      <c r="G35" s="77"/>
-      <c r="H35" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="I35" s="87" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="A36" s="135"/>
-      <c r="B36" s="103"/>
-      <c r="C36" s="105"/>
-      <c r="D36" s="39" t="s">
-        <v>100</v>
-      </c>
-      <c r="E36" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="F36" s="40" t="s">
-        <v>72</v>
-      </c>
-      <c r="G36" s="95"/>
+      <c r="G36" s="83"/>
       <c r="H36" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I36" s="107"/>
+      <c r="I36" s="119"/>
     </row>
     <row r="37" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="135"/>
-      <c r="B37" s="80"/>
-      <c r="C37" s="106"/>
-      <c r="D37" s="136"/>
+      <c r="A37" s="89"/>
+      <c r="B37" s="91"/>
+      <c r="C37" s="117"/>
+      <c r="D37" s="49"/>
       <c r="E37" s="20" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F37" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="G37" s="78"/>
+        <v>95</v>
+      </c>
+      <c r="G37" s="75"/>
       <c r="H37" s="33"/>
-      <c r="I37" s="88"/>
+      <c r="I37" s="120"/>
     </row>
     <row r="38" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="135"/>
+      <c r="A38" s="89"/>
       <c r="B38" s="63">
         <v>20</v>
       </c>
@@ -2133,27 +2130,27 @@
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="13" t="s">
-        <v>76</v>
+        <v>110</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A39" s="117"/>
-      <c r="B39" s="102" t="s">
-        <v>86</v>
-      </c>
-      <c r="C39" s="102"/>
-      <c r="D39" s="102"/>
-      <c r="E39" s="102"/>
-      <c r="F39" s="102"/>
-      <c r="G39" s="102"/>
-      <c r="H39" s="102"/>
-      <c r="I39" s="131"/>
+      <c r="A39" s="73"/>
+      <c r="B39" s="81" t="s">
+        <v>84</v>
+      </c>
+      <c r="C39" s="81"/>
+      <c r="D39" s="81"/>
+      <c r="E39" s="81"/>
+      <c r="F39" s="81"/>
+      <c r="G39" s="81"/>
+      <c r="H39" s="81"/>
+      <c r="I39" s="82"/>
     </row>
     <row r="40" spans="1:9" s="14" customFormat="1" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="117"/>
+      <c r="A40" s="73"/>
       <c r="B40" s="16"/>
       <c r="C40" s="15">
         <f>COUNTIF(C4:C38, "&lt;&gt;")</f>
@@ -2185,36 +2182,100 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A41" s="117"/>
-      <c r="B41" s="102" t="str">
+      <c r="A41" s="73"/>
+      <c r="B41" s="81" t="str">
         <f>SUM(C40:I40) &amp; " Total Races (Prior to Breeders' Cup Weekend)"</f>
         <v>94 Total Races (Prior to Breeders' Cup Weekend)</v>
       </c>
-      <c r="C41" s="102"/>
-      <c r="D41" s="102"/>
-      <c r="E41" s="102"/>
-      <c r="F41" s="102"/>
-      <c r="G41" s="102"/>
-      <c r="H41" s="102"/>
-      <c r="I41" s="102"/>
+      <c r="C41" s="81"/>
+      <c r="D41" s="81"/>
+      <c r="E41" s="81"/>
+      <c r="F41" s="81"/>
+      <c r="G41" s="81"/>
+      <c r="H41" s="81"/>
+      <c r="I41" s="81"/>
     </row>
     <row r="42" spans="1:9" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="117"/>
-      <c r="B42" s="126" t="s">
-        <v>84</v>
-      </c>
-      <c r="C42" s="126"/>
-      <c r="D42" s="126"/>
-      <c r="E42" s="127"/>
-      <c r="F42" s="128" t="s">
-        <v>85</v>
-      </c>
-      <c r="G42" s="129"/>
-      <c r="H42" s="129"/>
-      <c r="I42" s="130"/>
+      <c r="A42" s="73"/>
+      <c r="B42" s="76" t="s">
+        <v>82</v>
+      </c>
+      <c r="C42" s="76"/>
+      <c r="D42" s="76"/>
+      <c r="E42" s="77"/>
+      <c r="F42" s="78" t="s">
+        <v>83</v>
+      </c>
+      <c r="G42" s="79"/>
+      <c r="H42" s="79"/>
+      <c r="I42" s="80"/>
     </row>
   </sheetData>
   <mergeCells count="80">
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="G12:G13"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="I12:I13"/>
+    <mergeCell ref="H20:H21"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="G35:G37"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="C35:C37"/>
+    <mergeCell ref="I35:I37"/>
+    <mergeCell ref="H16:H18"/>
+    <mergeCell ref="G16:G18"/>
+    <mergeCell ref="F16:F18"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="F24:F26"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="I30:I31"/>
+    <mergeCell ref="G30:G31"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="I24:I26"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="H27:H28"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="H30:H31"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="F30:F31"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="A39:A42"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="B9:B10"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="F4:F5"/>
@@ -2231,70 +2292,6 @@
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="D20:D21"/>
     <mergeCell ref="H4:H5"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="E16:E18"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="F30:F31"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="A39:A42"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="I30:I31"/>
-    <mergeCell ref="G30:G31"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="H12:H13"/>
-    <mergeCell ref="I12:I13"/>
-    <mergeCell ref="H20:H21"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="B41:I41"/>
-    <mergeCell ref="G35:G37"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="C35:C37"/>
-    <mergeCell ref="I35:I37"/>
-    <mergeCell ref="H16:H18"/>
-    <mergeCell ref="G16:G18"/>
-    <mergeCell ref="F16:F18"/>
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="F24:F26"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="I24:I26"/>
-    <mergeCell ref="G27:G28"/>
-    <mergeCell ref="H27:H28"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="H30:H31"/>
-    <mergeCell ref="I20:I21"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="G12:G13"/>
-    <mergeCell ref="D14:D15"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="51" fitToHeight="10" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>